<commit_message>
feat: add JJJ batch source inversion data workflow
- add JJJ abnormal-high extraction and hourly workbook merge scripts
- support unit-stripped pollutant names and skip-list matching for JJJ pollutants
- make recent leak batch runner use an explicit abnormal event workbook
- update batch runner to call the JJJ extractor and refresh PINN input paths per event
- record actual sites/concentration/wind paths in batch summaries
- improve recurrent PDE speed settings and source initialization behavior
- fix diffusion GIF boundary extrapolation artifacts by masking outside valid PDE domain
</commit_message>
<xml_diff>
--- a/data/jjj/concentration.xlsx
+++ b/data/jjj/concentration.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -433,603 +433,309 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>K2站点（渤海十路边界点位）</t>
+          <t>M1站点（临港西部控制点位）</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>K3站点（汉江道边界点位）</t>
+          <t>M2站点（临港东部控制点位）</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>M1站点（临港西部控制点位）</t>
+          <t>M3站点（临港南部控制点位）</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>M2站点（临港东部控制点位）</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>M3站点（临港南部控制点位）</t>
+          <t>TARGET_POLLUTANT</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46117.75</v>
+        <v>46166.04166666666</v>
       </c>
       <c r="B2" t="n">
-        <v>0.28</v>
+        <v>0.06</v>
       </c>
       <c r="C2" t="n">
-        <v>18.17</v>
+        <v>4.35</v>
       </c>
       <c r="D2" t="n">
-        <v>2.51</v>
+        <v>4.12</v>
       </c>
       <c r="E2" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0.57</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0.16</v>
+        <v>3.08</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1-戊烯</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46117.79166666666</v>
+        <v>46166.08333333334</v>
       </c>
       <c r="B3" t="n">
-        <v>0.29</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="C3" t="n">
-        <v>18.04</v>
+        <v>5.06</v>
       </c>
       <c r="D3" t="n">
-        <v>2.51</v>
+        <v>3.41</v>
       </c>
       <c r="E3" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.17</v>
+        <v>3.48</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1-戊烯</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46117.83333333334</v>
+        <v>46166.125</v>
       </c>
       <c r="B4" t="n">
-        <v>468.3</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="C4" t="n">
-        <v>18.62</v>
+        <v>11.83</v>
       </c>
       <c r="D4" t="n">
-        <v>2.51</v>
+        <v>4.87</v>
       </c>
       <c r="E4" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0.48</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.17</v>
+        <v>3.95</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>1-戊烯</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46117.875</v>
+        <v>46166.16666666666</v>
       </c>
       <c r="B5" t="n">
-        <v>161.04</v>
+        <v>0.17</v>
       </c>
       <c r="C5" t="n">
-        <v>18.1</v>
+        <v>6.94</v>
       </c>
       <c r="D5" t="n">
-        <v>2.51</v>
+        <v>4.58</v>
       </c>
       <c r="E5" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0.43</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.2</v>
+        <v>4.04</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>1-戊烯</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46117.91666666666</v>
+        <v>46166.20833333334</v>
       </c>
       <c r="B6" t="n">
-        <v>25.39</v>
+        <v>0.13</v>
       </c>
       <c r="C6" t="n">
-        <v>18.1</v>
+        <v>5.81</v>
       </c>
       <c r="D6" t="n">
-        <v>2.51</v>
+        <v>4.62</v>
       </c>
       <c r="E6" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0.2</v>
+        <v>3.81</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1-戊烯</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46117.95833333334</v>
+        <v>46166.25</v>
       </c>
       <c r="B7" t="n">
-        <v>266.97</v>
+        <v>0.09</v>
       </c>
       <c r="C7" t="n">
-        <v>18.1</v>
+        <v>35.13</v>
       </c>
       <c r="D7" t="n">
-        <v>2.48</v>
+        <v>4.56</v>
       </c>
       <c r="E7" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0.24</v>
+        <v>4.04</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1-戊烯</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46118</v>
+        <v>46166.29166666666</v>
       </c>
       <c r="B8" t="n">
-        <v>288.46</v>
+        <v>0.23</v>
       </c>
       <c r="C8" t="n">
-        <v>17.97</v>
+        <v>658.88</v>
       </c>
       <c r="D8" t="n">
-        <v>2.48</v>
+        <v>5.23</v>
       </c>
       <c r="E8" t="n">
-        <v>0.19</v>
-      </c>
-      <c r="F8" t="n">
-        <v>1.32</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.28</v>
+        <v>3.92</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>1-戊烯</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46118.04166666666</v>
+        <v>46166.33333333334</v>
       </c>
       <c r="B9" t="n">
-        <v>107.32</v>
+        <v>0.29</v>
       </c>
       <c r="C9" t="n">
-        <v>17.91</v>
+        <v>95.83</v>
       </c>
       <c r="D9" t="n">
-        <v>2.29</v>
+        <v>5.8</v>
       </c>
       <c r="E9" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0.27</v>
+        <v>5.51</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1-戊烯</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46118.08333333334</v>
+        <v>46166.375</v>
       </c>
       <c r="B10" t="n">
-        <v>278.49</v>
+        <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>15.94</v>
+        <v>241.48</v>
       </c>
       <c r="D10" t="n">
-        <v>1.51</v>
+        <v>6.56</v>
       </c>
       <c r="E10" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0.23</v>
+        <v>6.81</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>1-戊烯</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46118.125</v>
+        <v>46166.41666666666</v>
       </c>
       <c r="B11" t="n">
-        <v>12.91</v>
+        <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>17.59</v>
+        <v>11.28</v>
       </c>
       <c r="D11" t="n">
-        <v>2.09</v>
+        <v>5.33</v>
       </c>
       <c r="E11" t="n">
-        <v>0.19</v>
-      </c>
-      <c r="F11" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="G11" t="n">
-        <v>46.32</v>
+        <v>5.97</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>1-戊烯</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46118.16666666666</v>
+        <v>46166.45833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>184.47</v>
+        <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>17.68</v>
+        <v>97.26000000000001</v>
       </c>
       <c r="D12" t="n">
-        <v>1.87</v>
+        <v>5.18</v>
       </c>
       <c r="E12" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="F12" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G12" t="n">
-        <v>0.68</v>
+        <v>4.63</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>1-戊烯</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46118.20833333334</v>
+        <v>46166.5</v>
       </c>
       <c r="B13" t="n">
-        <v>133.45</v>
+        <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>17.26</v>
+        <v>43.98</v>
       </c>
       <c r="D13" t="n">
-        <v>2.29</v>
+        <v>4.69</v>
       </c>
       <c r="E13" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="F13" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0.5600000000000001</v>
+        <v>4.11</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>1-戊烯</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46118.25</v>
+        <v>46166.54166666666</v>
       </c>
       <c r="B14" t="n">
-        <v>1.66</v>
+        <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>17.97</v>
+        <v>32.04</v>
       </c>
       <c r="D14" t="n">
-        <v>2.22</v>
+        <v>2.99</v>
       </c>
       <c r="E14" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="F14" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G14" t="n">
-        <v>12.78</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="n">
-        <v>46118.29166666666</v>
-      </c>
-      <c r="B15" t="n">
-        <v>45.83</v>
-      </c>
-      <c r="C15" t="n">
-        <v>17.78</v>
-      </c>
-      <c r="D15" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="F15" t="n">
-        <v>0.41</v>
-      </c>
-      <c r="G15" t="n">
-        <v>3.71</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="n">
-        <v>46118.33333333334</v>
-      </c>
-      <c r="B16" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="C16" t="n">
-        <v>18.26</v>
-      </c>
-      <c r="D16" t="n">
-        <v>2.45</v>
-      </c>
-      <c r="E16" t="n">
-        <v>0.44</v>
-      </c>
-      <c r="F16" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="G16" t="n">
-        <v>4.98</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="n">
-        <v>46118.375</v>
-      </c>
-      <c r="B17" t="n">
-        <v>0.89</v>
-      </c>
-      <c r="C17" t="n">
-        <v>18.3</v>
-      </c>
-      <c r="D17" t="n">
-        <v>2.48</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F17" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0.22</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="n">
-        <v>46118.41666666666</v>
-      </c>
-      <c r="B18" t="n">
-        <v>8.07</v>
-      </c>
-      <c r="C18" t="n">
-        <v>17.91</v>
-      </c>
-      <c r="D18" t="n">
-        <v>2.48</v>
-      </c>
-      <c r="E18" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="F18" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0.17</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="n">
-        <v>46118.45833333334</v>
-      </c>
-      <c r="B19" t="n">
-        <v>2.55</v>
-      </c>
-      <c r="C19" t="n">
-        <v>18.07</v>
-      </c>
-      <c r="D19" t="n">
-        <v>2.48</v>
-      </c>
-      <c r="E19" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="F19" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="G19" t="n">
-        <v>0.28</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="n">
-        <v>46118.5</v>
-      </c>
-      <c r="B20" t="n">
-        <v>0.48</v>
-      </c>
-      <c r="C20" t="n">
-        <v>18.39</v>
-      </c>
-      <c r="D20" t="n">
-        <v>2.42</v>
-      </c>
-      <c r="E20" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="F20" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="G20" t="n">
-        <v>0.31</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="n">
-        <v>46118.54166666666</v>
-      </c>
-      <c r="B21" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="C21" t="n">
-        <v>17.72</v>
-      </c>
-      <c r="D21" t="n">
-        <v>2.38</v>
-      </c>
-      <c r="E21" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="F21" t="n">
-        <v>0.41</v>
-      </c>
-      <c r="G21" t="n">
-        <v>0.23</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="n">
-        <v>46118.58333333334</v>
-      </c>
-      <c r="B22" t="n">
-        <v>0.66</v>
-      </c>
-      <c r="C22" t="n">
-        <v>17.62</v>
-      </c>
-      <c r="D22" t="n">
-        <v>2.35</v>
-      </c>
-      <c r="E22" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="F22" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="G22" t="n">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="1" t="n">
-        <v>46118.625</v>
-      </c>
-      <c r="B23" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="C23" t="n">
-        <v>17.72</v>
-      </c>
-      <c r="D23" t="n">
-        <v>2.35</v>
-      </c>
-      <c r="E23" t="n">
-        <v>6.26</v>
-      </c>
-      <c r="F23" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="G23" t="n">
-        <v>0.35</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="n">
-        <v>46118.66666666666</v>
-      </c>
-      <c r="B24" t="n">
-        <v>0.41</v>
-      </c>
-      <c r="C24" t="n">
-        <v>17.68</v>
-      </c>
-      <c r="D24" t="n">
-        <v>2.35</v>
-      </c>
-      <c r="E24" t="n">
-        <v>10.73</v>
-      </c>
-      <c r="F24" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="G24" t="n">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="1" t="n">
-        <v>46118.70833333334</v>
-      </c>
-      <c r="B25" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="C25" t="n">
-        <v>17.59</v>
-      </c>
-      <c r="D25" t="n">
-        <v>2.32</v>
-      </c>
-      <c r="E25" t="n">
-        <v>35.41</v>
-      </c>
-      <c r="F25" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="G25" t="n">
-        <v>0.19</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="1" t="n">
-        <v>46118.75</v>
-      </c>
-      <c r="B26" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="C26" t="n">
-        <v>17.3</v>
-      </c>
-      <c r="D26" t="n">
-        <v>2.29</v>
-      </c>
-      <c r="E26" t="n">
-        <v>64.7</v>
-      </c>
-      <c r="F26" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="G26" t="n">
-        <v>0.22</v>
+        <v>3.6</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>1-戊烯</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: make batch inversion refresh inputs per event
- support switching recent leak batch runs between JJJ and SHSH-JS data sources
- parse actual extracted concentration/wind/sites paths before launching PINN
- update PINN config paths and target pollutant for each leak event
- add JJJ abnormal-high extraction and hourly workbook merge utilities
- clean pollutant units and improve skip-pollutant matching for JJJ outputs
- fix diffusion GIF valid-domain cropping and boundary visualization artifacts
</commit_message>
<xml_diff>
--- a/data/jjj/concentration.xlsx
+++ b/data/jjj/concentration.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:M14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -428,25 +428,60 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>H1站点（装备制造区域点位）</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>H2站点（罐区区域点位）</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>H3站点（海河道区域点位）</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>H4站点（粮油区域点位）</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>H5站点（淮河道区域点位）</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>K1站点（园区中心点位）</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>K2站点（渤海十路边界点位）</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>K3站点（汉江道边界点位）</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
         <is>
           <t>M1站点（临港西部控制点位）</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>M2站点（临港东部控制点位）</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>M3站点（临港南部控制点位）</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>TARGET_POLLUTANT</t>
         </is>
@@ -454,287 +489,560 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46166.04166666666</v>
+        <v>46157.04166666666</v>
       </c>
       <c r="B2" t="n">
-        <v>0.06</v>
+        <v>16.9</v>
       </c>
       <c r="C2" t="n">
-        <v>4.35</v>
+        <v>77.2</v>
       </c>
       <c r="D2" t="n">
-        <v>4.12</v>
+        <v>3.4</v>
       </c>
       <c r="E2" t="n">
-        <v>3.08</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>1-戊烯</t>
+        <v>0.2</v>
+      </c>
+      <c r="F2" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="G2" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="I2" t="n">
+        <v>21.66</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>6.22</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>乙苯</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46166.08333333334</v>
+        <v>46157.08333333334</v>
       </c>
       <c r="B3" t="n">
-        <v>0.07000000000000001</v>
+        <v>14.3</v>
       </c>
       <c r="C3" t="n">
-        <v>5.06</v>
+        <v>83.7</v>
       </c>
       <c r="D3" t="n">
-        <v>3.41</v>
+        <v>3.5</v>
       </c>
       <c r="E3" t="n">
-        <v>3.48</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>1-戊烯</t>
+        <v>0.4</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="G3" t="n">
+        <v>4.31</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="I3" t="n">
+        <v>22.94</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>乙苯</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46166.125</v>
+        <v>46157.125</v>
       </c>
       <c r="B4" t="n">
-        <v>0.07000000000000001</v>
+        <v>6.7</v>
       </c>
       <c r="C4" t="n">
-        <v>11.83</v>
+        <v>97.5</v>
       </c>
       <c r="D4" t="n">
-        <v>4.87</v>
+        <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>3.95</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>1-戊烯</t>
+        <v>0.2</v>
+      </c>
+      <c r="F4" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="I4" t="n">
+        <v>23.37</v>
+      </c>
+      <c r="J4" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>乙苯</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46166.16666666666</v>
+        <v>46157.16666666666</v>
       </c>
       <c r="B5" t="n">
-        <v>0.17</v>
+        <v>4.4</v>
       </c>
       <c r="C5" t="n">
-        <v>6.94</v>
+        <v>62</v>
       </c>
       <c r="D5" t="n">
-        <v>4.58</v>
+        <v>1.8</v>
       </c>
       <c r="E5" t="n">
-        <v>4.04</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>1-戊烯</t>
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G5" t="n">
+        <v>4.28</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="I5" t="n">
+        <v>22.47</v>
+      </c>
+      <c r="J5" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>乙苯</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46166.20833333334</v>
+        <v>46157.20833333334</v>
       </c>
       <c r="B6" t="n">
-        <v>0.13</v>
+        <v>2.8</v>
       </c>
       <c r="C6" t="n">
-        <v>5.81</v>
+        <v>172</v>
       </c>
       <c r="D6" t="n">
-        <v>4.62</v>
+        <v>1.3</v>
       </c>
       <c r="E6" t="n">
-        <v>3.81</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>1-戊烯</t>
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G6" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="I6" t="n">
+        <v>22.61</v>
+      </c>
+      <c r="J6" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>乙苯</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46166.25</v>
+        <v>46157.25</v>
       </c>
       <c r="B7" t="n">
-        <v>0.09</v>
+        <v>3.7</v>
       </c>
       <c r="C7" t="n">
-        <v>35.13</v>
+        <v>55</v>
       </c>
       <c r="D7" t="n">
-        <v>4.56</v>
+        <v>0.9</v>
       </c>
       <c r="E7" t="n">
-        <v>4.04</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>1-戊烯</t>
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="I7" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>乙苯</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46166.29166666666</v>
+        <v>46157.29166666666</v>
       </c>
       <c r="B8" t="n">
-        <v>0.23</v>
+        <v>2.9</v>
       </c>
       <c r="C8" t="n">
-        <v>658.88</v>
+        <v>591.5</v>
       </c>
       <c r="D8" t="n">
-        <v>5.23</v>
+        <v>0.4</v>
       </c>
       <c r="E8" t="n">
-        <v>3.92</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>1-戊烯</t>
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="I8" t="n">
+        <v>22.18</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>乙苯</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46166.33333333334</v>
+        <v>46157.33333333334</v>
       </c>
       <c r="B9" t="n">
-        <v>0.29</v>
+        <v>3.7</v>
       </c>
       <c r="C9" t="n">
-        <v>95.83</v>
+        <v>496.1</v>
       </c>
       <c r="D9" t="n">
-        <v>5.8</v>
+        <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>5.51</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>1-戊烯</t>
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="I9" t="n">
+        <v>22.61</v>
+      </c>
+      <c r="J9" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>乙苯</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46166.375</v>
+        <v>46157.375</v>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>5.2</v>
       </c>
       <c r="C10" t="n">
-        <v>241.48</v>
+        <v>100.8</v>
       </c>
       <c r="D10" t="n">
-        <v>6.56</v>
+        <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>6.81</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>1-戊烯</t>
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="I10" t="n">
+        <v>23.65</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>乙苯</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46166.41666666666</v>
+        <v>46157.41666666666</v>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>3.6</v>
       </c>
       <c r="C11" t="n">
-        <v>11.28</v>
+        <v>35.7</v>
       </c>
       <c r="D11" t="n">
-        <v>5.33</v>
+        <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>5.97</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>1-戊烯</t>
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="I11" t="n">
+        <v>22.56</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>乙苯</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46166.45833333334</v>
+        <v>46157.45833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>2.1</v>
       </c>
       <c r="C12" t="n">
-        <v>97.26000000000001</v>
+        <v>12.3</v>
       </c>
       <c r="D12" t="n">
-        <v>5.18</v>
+        <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>4.63</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>1-戊烯</t>
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="I12" t="n">
+        <v>22.18</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>乙苯</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46166.5</v>
+        <v>46157.5</v>
       </c>
       <c r="B13" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C13" t="n">
-        <v>43.98</v>
+        <v>15</v>
       </c>
       <c r="D13" t="n">
-        <v>4.69</v>
+        <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>4.11</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>1-戊烯</t>
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="I13" t="n">
+        <v>22.32</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>乙苯</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46166.54166666666</v>
+        <v>46157.54166666666</v>
       </c>
       <c r="B14" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C14" t="n">
-        <v>32.04</v>
+        <v>28</v>
       </c>
       <c r="D14" t="n">
-        <v>2.99</v>
+        <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>1-戊烯</t>
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="H14" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="I14" t="n">
+        <v>21.09</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="L14" t="n">
+        <v>48.82</v>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>乙苯</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: align recurrent plume timing and slow diffusion GIF
- store the initial release at the source before advection
- use symmetric source injection across each transport interval
- evaluate source strength at both substep endpoints
- make diffusion GIF playback speed configurable and reduce it to 2 fps
- add regression tests for source-centered initial fields
</commit_message>
<xml_diff>
--- a/data/jjj/concentration.xlsx
+++ b/data/jjj/concentration.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -428,60 +428,25 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>H1站点（装备制造区域点位）</t>
+          <t>K1站点（园区中心点位）</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>H2站点（罐区区域点位）</t>
+          <t>M1站点（临港西部控制点位）</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>H3站点（海河道区域点位）</t>
+          <t>M2站点（临港东部控制点位）</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>H4站点（粮油区域点位）</t>
+          <t>M3站点（临港南部控制点位）</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
-        <is>
-          <t>H5站点（淮河道区域点位）</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>K1站点（园区中心点位）</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>K2站点（渤海十路边界点位）</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>K3站点（汉江道边界点位）</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>M1站点（临港西部控制点位）</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>M2站点（临港东部控制点位）</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>M3站点（临港南部控制点位）</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
         <is>
           <t>TARGET_POLLUTANT</t>
         </is>
@@ -489,560 +454,287 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46157.04166666666</v>
+        <v>46165.5</v>
       </c>
       <c r="B2" t="n">
-        <v>16.9</v>
+        <v>3.28</v>
       </c>
       <c r="C2" t="n">
-        <v>77.2</v>
+        <v>65.59</v>
       </c>
       <c r="D2" t="n">
-        <v>3.4</v>
+        <v>2.33</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F2" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="G2" t="n">
-        <v>3.97</v>
-      </c>
-      <c r="H2" t="n">
-        <v>1.28</v>
-      </c>
-      <c r="I2" t="n">
-        <v>21.66</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>6.22</v>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>乙苯</t>
+        <v>2.52</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>异戊烷</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46157.08333333334</v>
+        <v>46165.54166666666</v>
       </c>
       <c r="B3" t="n">
-        <v>14.3</v>
+        <v>3.2</v>
       </c>
       <c r="C3" t="n">
-        <v>83.7</v>
+        <v>162.43</v>
       </c>
       <c r="D3" t="n">
-        <v>3.5</v>
+        <v>2.31</v>
       </c>
       <c r="E3" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="F3" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="G3" t="n">
-        <v>4.31</v>
-      </c>
-      <c r="H3" t="n">
-        <v>1.18</v>
-      </c>
-      <c r="I3" t="n">
-        <v>22.94</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>乙苯</t>
+        <v>1.97</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>异戊烷</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46157.125</v>
+        <v>46165.58333333334</v>
       </c>
       <c r="B4" t="n">
-        <v>6.7</v>
+        <v>3.18</v>
       </c>
       <c r="C4" t="n">
-        <v>97.5</v>
+        <v>1.56</v>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>4.55</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F4" t="n">
-        <v>7.4</v>
-      </c>
-      <c r="G4" t="n">
-        <v>1.73</v>
-      </c>
-      <c r="H4" t="n">
-        <v>1.18</v>
-      </c>
-      <c r="I4" t="n">
-        <v>23.37</v>
-      </c>
-      <c r="J4" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>乙苯</t>
+        <v>1.62</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>异戊烷</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46157.16666666666</v>
+        <v>46165.625</v>
       </c>
       <c r="B5" t="n">
-        <v>4.4</v>
+        <v>1.88</v>
       </c>
       <c r="C5" t="n">
-        <v>62</v>
+        <v>68.73</v>
       </c>
       <c r="D5" t="n">
-        <v>1.8</v>
+        <v>1.66</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="G5" t="n">
-        <v>4.28</v>
-      </c>
-      <c r="H5" t="n">
-        <v>1.52</v>
-      </c>
-      <c r="I5" t="n">
-        <v>22.47</v>
-      </c>
-      <c r="J5" t="n">
-        <v>3.78</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>乙苯</t>
+        <v>0.91</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>异戊烷</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46157.20833333334</v>
+        <v>46165.66666666666</v>
       </c>
       <c r="B6" t="n">
-        <v>2.8</v>
+        <v>2.27</v>
       </c>
       <c r="C6" t="n">
-        <v>172</v>
+        <v>33.59</v>
       </c>
       <c r="D6" t="n">
-        <v>1.3</v>
+        <v>2.12</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G6" t="n">
-        <v>3.16</v>
-      </c>
-      <c r="H6" t="n">
-        <v>1.71</v>
-      </c>
-      <c r="I6" t="n">
-        <v>22.61</v>
-      </c>
-      <c r="J6" t="n">
-        <v>4.55</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>乙苯</t>
+        <v>1.16</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>异戊烷</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46157.25</v>
+        <v>46165.70833333334</v>
       </c>
       <c r="B7" t="n">
-        <v>3.7</v>
+        <v>2.36</v>
       </c>
       <c r="C7" t="n">
-        <v>55</v>
+        <v>8.56</v>
       </c>
       <c r="D7" t="n">
-        <v>0.9</v>
+        <v>1.95</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="H7" t="n">
-        <v>1.47</v>
-      </c>
-      <c r="I7" t="n">
-        <v>22.8</v>
-      </c>
-      <c r="J7" t="n">
-        <v>1.23</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>乙苯</t>
+        <v>1.1</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>异戊烷</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46157.29166666666</v>
+        <v>46165.75</v>
       </c>
       <c r="B8" t="n">
-        <v>2.9</v>
+        <v>1.64</v>
       </c>
       <c r="C8" t="n">
-        <v>591.5</v>
+        <v>597.92</v>
       </c>
       <c r="D8" t="n">
-        <v>0.4</v>
+        <v>1.15</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G8" t="n">
-        <v>1.18</v>
-      </c>
-      <c r="H8" t="n">
-        <v>1.23</v>
-      </c>
-      <c r="I8" t="n">
-        <v>22.18</v>
-      </c>
-      <c r="J8" t="n">
-        <v>1.26</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0.19</v>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>乙苯</t>
+        <v>0.99</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>异戊烷</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46157.33333333334</v>
+        <v>46165.79166666666</v>
       </c>
       <c r="B9" t="n">
-        <v>3.7</v>
+        <v>1.44</v>
       </c>
       <c r="C9" t="n">
-        <v>496.1</v>
+        <v>2.71</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>1.87</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="H9" t="n">
-        <v>1.14</v>
-      </c>
-      <c r="I9" t="n">
-        <v>22.61</v>
-      </c>
-      <c r="J9" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0.19</v>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>乙苯</t>
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>异戊烷</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46157.375</v>
+        <v>46165.83333333334</v>
       </c>
       <c r="B10" t="n">
-        <v>5.2</v>
+        <v>1.76</v>
       </c>
       <c r="C10" t="n">
-        <v>100.8</v>
+        <v>28.47</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>1.76</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="I10" t="n">
-        <v>23.65</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>乙苯</t>
+        <v>0.98</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>异戊烷</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46157.41666666666</v>
+        <v>46165.875</v>
       </c>
       <c r="B11" t="n">
-        <v>3.6</v>
+        <v>2.01</v>
       </c>
       <c r="C11" t="n">
-        <v>35.7</v>
+        <v>0.95</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>1.94</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="H11" t="n">
-        <v>1.14</v>
-      </c>
-      <c r="I11" t="n">
-        <v>22.56</v>
-      </c>
-      <c r="J11" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>乙苯</t>
+        <v>0.92</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>异戊烷</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46157.45833333334</v>
+        <v>46165.91666666666</v>
       </c>
       <c r="B12" t="n">
-        <v>2.1</v>
+        <v>3.43</v>
       </c>
       <c r="C12" t="n">
-        <v>12.3</v>
+        <v>10.54</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>3.89</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="H12" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="I12" t="n">
-        <v>22.18</v>
-      </c>
-      <c r="J12" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="K12" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="L12" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>乙苯</t>
+        <v>2.82</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>异戊烷</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46157.5</v>
+        <v>46165.95833333334</v>
       </c>
       <c r="B13" t="n">
-        <v>3</v>
+        <v>4.88</v>
       </c>
       <c r="C13" t="n">
-        <v>15</v>
+        <v>2.69</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>4.52</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="H13" t="n">
-        <v>1.42</v>
-      </c>
-      <c r="I13" t="n">
-        <v>22.32</v>
-      </c>
-      <c r="J13" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="K13" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="L13" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>乙苯</t>
+        <v>2.79</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>异戊烷</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46157.54166666666</v>
+        <v>46166</v>
       </c>
       <c r="B14" t="n">
-        <v>4</v>
+        <v>5.29</v>
       </c>
       <c r="C14" t="n">
-        <v>28</v>
+        <v>4.06</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>5.02</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="H14" t="n">
-        <v>1.28</v>
-      </c>
-      <c r="I14" t="n">
-        <v>21.09</v>
-      </c>
-      <c r="J14" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="K14" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="L14" t="n">
-        <v>48.82</v>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>乙苯</t>
+        <v>3.44</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>异戊烷</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: streamline inversion outputs and improve monitor data workflow
- export hourly concentration fields and source coordinates for each inversion
- consolidate Q, training, station, and landscape diagnostics into diagnostics.xlsx
- merge source confidence metadata into result_quality_report.json
- replace duplicate confidence plots with a unified source confidence figure
- support manual pollutant filtering in batch inversion and abnormal extraction
- update JJJ extractors to read the combined multi-station workbook
- improve SHSH-JS and JJJ input path propagation between batch tasks
- update documentation and project status
</commit_message>
<xml_diff>
--- a/data/jjj/concentration.xlsx
+++ b/data/jjj/concentration.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -428,25 +428,65 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>H4站点（粮油区域点位）</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>H5站点（淮河道区域点位）</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>K1站点（园区中心点位）</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>K2站点（渤海十路边界点位）</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>K3站点（汉江道边界点位）</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
         <is>
           <t>M1站点（临港西部控制点位）</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>M2站点（临港东部控制点位）</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>M3站点（临港南部控制点位）</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Z1站点（渤海十路点位）</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Z2站点（辽河道点位）</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Z3站点（渤海十六路点位）</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Z4站点（渤海十八路点位）</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
         <is>
           <t>TARGET_POLLUTANT</t>
         </is>
@@ -454,287 +494,599 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46165.5</v>
+        <v>46145.79166666666</v>
       </c>
       <c r="B2" t="n">
-        <v>3.28</v>
+        <v>15.93</v>
       </c>
       <c r="C2" t="n">
-        <v>65.59</v>
+        <v>3.67</v>
       </c>
       <c r="D2" t="n">
-        <v>2.33</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>2.52</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>异戊烷</t>
+        <v>5.72</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>氨</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46165.54166666666</v>
+        <v>46145.83333333334</v>
       </c>
       <c r="B3" t="n">
-        <v>3.2</v>
+        <v>12.16</v>
       </c>
       <c r="C3" t="n">
-        <v>162.43</v>
+        <v>-1.75</v>
       </c>
       <c r="D3" t="n">
-        <v>2.31</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>1.97</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>异戊烷</t>
+        <v>7.62</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>氨</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46165.58333333334</v>
+        <v>46145.875</v>
       </c>
       <c r="B4" t="n">
-        <v>3.18</v>
+        <v>16.5</v>
       </c>
       <c r="C4" t="n">
-        <v>1.56</v>
+        <v>-4.59</v>
       </c>
       <c r="D4" t="n">
-        <v>4.55</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>1.62</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>异戊烷</t>
+        <v>21.57</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>氨</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46165.625</v>
+        <v>46145.91666666666</v>
       </c>
       <c r="B5" t="n">
-        <v>1.88</v>
+        <v>19.68</v>
       </c>
       <c r="C5" t="n">
-        <v>68.73</v>
+        <v>18.44</v>
       </c>
       <c r="D5" t="n">
-        <v>1.66</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>异戊烷</t>
+        <v>39.22</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>氨</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46165.66666666666</v>
+        <v>46145.95833333334</v>
       </c>
       <c r="B6" t="n">
-        <v>2.27</v>
+        <v>23.57</v>
       </c>
       <c r="C6" t="n">
-        <v>33.59</v>
+        <v>14.87</v>
       </c>
       <c r="D6" t="n">
-        <v>2.12</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>1.16</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>异戊烷</t>
+        <v>9.92</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>氨</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46165.70833333334</v>
+        <v>46146</v>
       </c>
       <c r="B7" t="n">
-        <v>2.36</v>
+        <v>24.3</v>
       </c>
       <c r="C7" t="n">
-        <v>8.56</v>
+        <v>181.16</v>
       </c>
       <c r="D7" t="n">
-        <v>1.95</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>异戊烷</t>
+        <v>11.06</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>氨</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46165.75</v>
+        <v>46146.04166666666</v>
       </c>
       <c r="B8" t="n">
-        <v>1.64</v>
+        <v>23.66</v>
       </c>
       <c r="C8" t="n">
-        <v>597.92</v>
+        <v>1078.66</v>
       </c>
       <c r="D8" t="n">
-        <v>1.15</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>0.99</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>异戊烷</t>
+        <v>10.01</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>氨</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46165.79166666666</v>
+        <v>46146.08333333334</v>
       </c>
       <c r="B9" t="n">
-        <v>1.44</v>
+        <v>20.39</v>
       </c>
       <c r="C9" t="n">
-        <v>2.71</v>
+        <v>234.51</v>
       </c>
       <c r="D9" t="n">
-        <v>1.87</v>
+        <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>异戊烷</t>
+        <v>12.75</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>氨</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46165.83333333334</v>
+        <v>46146.125</v>
       </c>
       <c r="B10" t="n">
-        <v>1.76</v>
+        <v>20.75</v>
       </c>
       <c r="C10" t="n">
-        <v>28.47</v>
+        <v>118.88</v>
       </c>
       <c r="D10" t="n">
-        <v>1.76</v>
+        <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>异戊烷</t>
+        <v>11.56</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>氨</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46165.875</v>
+        <v>46146.16666666666</v>
       </c>
       <c r="B11" t="n">
-        <v>2.01</v>
+        <v>18.09</v>
       </c>
       <c r="C11" t="n">
-        <v>0.95</v>
+        <v>83.81</v>
       </c>
       <c r="D11" t="n">
-        <v>1.94</v>
+        <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>异戊烷</t>
+        <v>12.61</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>氨</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46165.91666666666</v>
+        <v>46146.20833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>3.43</v>
+        <v>18.6</v>
       </c>
       <c r="C12" t="n">
-        <v>10.54</v>
+        <v>65.05</v>
       </c>
       <c r="D12" t="n">
-        <v>3.89</v>
+        <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>2.82</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>异戊烷</t>
+        <v>12.39</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>氨</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46165.95833333334</v>
+        <v>46146.25</v>
       </c>
       <c r="B13" t="n">
-        <v>4.88</v>
+        <v>18.23</v>
       </c>
       <c r="C13" t="n">
-        <v>2.69</v>
+        <v>54.39</v>
       </c>
       <c r="D13" t="n">
-        <v>4.52</v>
+        <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>2.79</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>异戊烷</t>
+        <v>13.03</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>氨</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46166</v>
+        <v>46146.29166666666</v>
       </c>
       <c r="B14" t="n">
-        <v>5.29</v>
+        <v>17.52</v>
       </c>
       <c r="C14" t="n">
-        <v>4.06</v>
+        <v>43.87</v>
       </c>
       <c r="D14" t="n">
-        <v>5.02</v>
+        <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>3.44</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>异戊烷</t>
+        <v>11.21</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>氨</t>
         </is>
       </c>
     </row>

</xml_diff>